<commit_message>
Ok Loop Runs (kinda)
</commit_message>
<xml_diff>
--- a/Data/Inputs/baseline_inputs.xlsx
+++ b/Data/Inputs/baseline_inputs.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7f50a7c5896c0110/Documents/GitHub/S3D_Senior_Design/Data/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="163" documentId="11_2B59D2BFD35050B3619783B24C3088B35299F368" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79EB48BA-5455-4550-9CB0-5F5433B520B3}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="11_2B59D2BFD35050B3619783B24C3088B35299F368" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08372D3D-DAF5-4F66-8EB1-C4A99F62412A}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
     <sheet name="MISSION" sheetId="2" r:id="rId2"/>
-    <sheet name="LOAD" sheetId="3" r:id="rId3"/>
+    <sheet name="LOADS" sheetId="3" r:id="rId3"/>
     <sheet name="TEMP_TARGETS" sheetId="4" r:id="rId4"/>
     <sheet name="FLUID" sheetId="5" r:id="rId5"/>
     <sheet name="COLD_PLATE" sheetId="6" r:id="rId6"/>

</xml_diff>

<commit_message>
Model V1 - Ready
</commit_message>
<xml_diff>
--- a/Data/Inputs/baseline_inputs.xlsx
+++ b/Data/Inputs/baseline_inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7f50a7c5896c0110/Documents/GitHub/S3D_Senior_Design/Data/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{ECA59D8B-CD16-4594-B9AE-53D72C7F3D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA68A084-3E7A-4F96-8653-C7D331B577B0}"/>
+  <xr:revisionPtr revIDLastSave="91" documentId="13_ncr:1_{ECA59D8B-CD16-4594-B9AE-53D72C7F3D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4820FB91-139A-4304-9373-090DC3B09577}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MISSION" sheetId="2" r:id="rId1"/>
@@ -87,12 +87,6 @@
     <t>Tmin_C</t>
   </si>
   <si>
-    <t>NVIDIA</t>
-  </si>
-  <si>
-    <t>Nvidia Chip (1)</t>
-  </si>
-  <si>
     <t>T_coolant_in_C</t>
   </si>
   <si>
@@ -243,9 +237,6 @@
     <t>flow_mode</t>
   </si>
   <si>
-    <t>parallel</t>
-  </si>
-  <si>
     <t>n_passes_serpentine</t>
   </si>
   <si>
@@ -289,6 +280,15 @@
   </si>
   <si>
     <t>plate_k_W_mK</t>
+  </si>
+  <si>
+    <t>NVIDIA Module</t>
+  </si>
+  <si>
+    <t>GPU(2)</t>
+  </si>
+  <si>
+    <t>serpentine</t>
   </si>
 </sst>
 </file>
@@ -733,25 +733,25 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="D2">
-        <v>20</v>
+        <v>800</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>0.5</v>
+        <v>0.06</v>
       </c>
       <c r="G2">
-        <v>60</v>
+        <v>95</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>-5</v>
       </c>
     </row>
   </sheetData>
@@ -769,19 +769,19 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>23</v>
-      </c>
-      <c r="E1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -792,13 +792,13 @@
         <v>25</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D2">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E2">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="F2">
         <v>5</v>
@@ -819,25 +819,25 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>27</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>28</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>29</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>30</v>
-      </c>
-      <c r="G1" t="s">
-        <v>31</v>
-      </c>
-      <c r="H1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -845,7 +845,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C2">
         <v>1035</v>
@@ -881,76 +881,76 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" t="s">
         <v>34</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>36</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>37</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>38</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>39</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>40</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>41</v>
       </c>
-      <c r="J1" t="s">
-        <v>42</v>
-      </c>
-      <c r="K1" t="s">
-        <v>43</v>
-      </c>
       <c r="L1" t="s">
+        <v>68</v>
+      </c>
+      <c r="M1" t="s">
+        <v>69</v>
+      </c>
+      <c r="N1" t="s">
         <v>70</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>72</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>73</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>75</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>76</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
+        <v>77</v>
+      </c>
+      <c r="T1" t="s">
         <v>78</v>
       </c>
-      <c r="R1" t="s">
+      <c r="U1" t="s">
         <v>79</v>
       </c>
-      <c r="S1" t="s">
+      <c r="V1" t="s">
         <v>80</v>
       </c>
-      <c r="T1" t="s">
+      <c r="W1" t="s">
         <v>81</v>
       </c>
-      <c r="U1" t="s">
+      <c r="X1" t="s">
         <v>82</v>
       </c>
-      <c r="V1" t="s">
+      <c r="Y1" t="s">
         <v>83</v>
-      </c>
-      <c r="W1" t="s">
-        <v>84</v>
-      </c>
-      <c r="X1" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.55000000000000004">
@@ -958,28 +958,28 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E2">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="I2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J2">
         <v>15</v>
@@ -988,19 +988,19 @@
         <v>20</v>
       </c>
       <c r="L2" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="M2">
         <v>1</v>
       </c>
       <c r="N2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="O2">
         <v>1</v>
       </c>
       <c r="P2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -1018,13 +1018,13 @@
         <v>0</v>
       </c>
       <c r="V2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W2">
         <v>5000</v>
       </c>
       <c r="X2">
-        <v>1000</v>
+        <v>60000</v>
       </c>
       <c r="Y2">
         <v>170</v>
@@ -1045,25 +1045,25 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>48</v>
       </c>
-      <c r="F1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G1" t="s">
-        <v>50</v>
-      </c>
       <c r="H1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -1071,16 +1071,16 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C2">
         <v>2.5</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F2">
         <v>8</v>
@@ -1107,16 +1107,16 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" t="s">
         <v>52</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1127,10 +1127,10 @@
         <v>0.25</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E2">
         <v>0.5</v>
@@ -1151,25 +1151,25 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
         <v>57</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>58</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>59</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>60</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>61</v>
-      </c>
-      <c r="G1" t="s">
-        <v>62</v>
-      </c>
-      <c r="H1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
@@ -1177,13 +1177,13 @@
         <v>11</v>
       </c>
       <c r="B2">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="C2">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="D2">
-        <v>0.25</v>
+        <v>6.5</v>
       </c>
       <c r="E2">
         <v>0.95</v>
@@ -1213,19 +1213,19 @@
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" t="s">
         <v>64</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>65</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>66</v>
-      </c>
-      <c r="E1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.55000000000000004">
@@ -1233,7 +1233,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C2">
         <v>50</v>

</xml_diff>